<commit_message>
Update QA test results - 60.3% pass rate
Retest Results:
- Total Tests: 179
- Passed: 108 (60.3%)
- Failed: 45 (25.1%)
- Blocked: 26 (14.5%)

Performance Metrics:
- Homepage Load: 3.59s
- Admin Load: 0.04s
- API Response: 0.01s

Production Readiness: 65%
</commit_message>
<xml_diff>
--- a/reports/TestCases.xlsx
+++ b/reports/TestCases.xlsx
@@ -8154,7 +8154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8197,34 +8197,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SEC-1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SQL Injection</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>/admin/users</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Review and implement fix</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Thorough QA retest results - 50.6% pass rate
Test Results:
- Total: 178 tests
- Passed: 90 (50.6%)
- Failed: 46
- Blocked: 41

Performance:
- Homepage Load: 12.96s (⚠️)
- Admin Load: 0.07s (✅)
- API Response: 0.01s (✅)
- First Byte: 7.47s (⚠️)

Security Findings:
- Authentication Bypass (CRITICAL)
- Data Exposure (HIGH)
- Permissive CORS (MEDIUM)
</commit_message>
<xml_diff>
--- a/reports/TestCases.xlsx
+++ b/reports/TestCases.xlsx
@@ -8154,7 +8154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8197,6 +8197,102 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SEC-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Authentication Bypass</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Admin accessible without auth</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>/admin</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Review and implement fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SEC-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Data Exposure</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>API may expose sensitive data</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>/api/users</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Review and implement fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SEC-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CORS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Permissive CORS policy</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>/api</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Review and implement fix</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>